<commit_message>
buscador en la vista selectList, descripciones detalladas al dejar el mouse en porcentaje
</commit_message>
<xml_diff>
--- a/LISTAS/mi/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/mi/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45216</v>
+        <v>45217</v>
       </c>
     </row>
     <row r="2">
@@ -843,10 +843,8 @@
         </is>
       </c>
       <c r="C26" s="20" t="n"/>
-      <c r="D26" s="22" t="inlineStr">
-        <is>
-          <t>602.352</t>
-        </is>
+      <c r="D26" s="22" t="n">
+        <v>542.1168</v>
       </c>
       <c r="E26" s="23" t="n"/>
       <c r="F26" s="23" t="n"/>
@@ -864,10 +862,8 @@
         </is>
       </c>
       <c r="C27" s="20" t="n"/>
-      <c r="D27" s="22" t="inlineStr">
-        <is>
-          <t>700.0</t>
-        </is>
+      <c r="D27" s="22" t="n">
+        <v>630</v>
       </c>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="n"/>
@@ -885,10 +881,8 @@
         </is>
       </c>
       <c r="C28" s="20" t="n"/>
-      <c r="D28" s="22" t="inlineStr">
-        <is>
-          <t>709.045</t>
-        </is>
+      <c r="D28" s="22" t="n">
+        <v>638.1405</v>
       </c>
       <c r="E28" s="23" t="n"/>
       <c r="F28" s="23" t="n"/>
@@ -906,10 +900,8 @@
         </is>
       </c>
       <c r="C29" s="20" t="n"/>
-      <c r="D29" s="22" t="inlineStr">
-        <is>
-          <t>1225.63</t>
-        </is>
+      <c r="D29" s="22" t="n">
+        <v>1103.067</v>
       </c>
       <c r="E29" s="23" t="n"/>
       <c r="F29" s="23" t="n"/>
@@ -927,10 +919,8 @@
         </is>
       </c>
       <c r="C30" s="20" t="n"/>
-      <c r="D30" s="22" t="inlineStr">
-        <is>
-          <t>1512.193</t>
-        </is>
+      <c r="D30" s="22" t="n">
+        <v>1360.9737</v>
       </c>
       <c r="E30" s="23" t="n"/>
       <c r="F30" s="23" t="n"/>
@@ -948,10 +938,8 @@
         </is>
       </c>
       <c r="C31" s="20" t="n"/>
-      <c r="D31" s="22" t="inlineStr">
-        <is>
-          <t>2005.801</t>
-        </is>
+      <c r="D31" s="22" t="n">
+        <v>1805.2209</v>
       </c>
       <c r="E31" s="23" t="n"/>
       <c r="F31" s="23" t="n"/>
@@ -969,10 +957,8 @@
         </is>
       </c>
       <c r="C32" s="20" t="n"/>
-      <c r="D32" s="22" t="inlineStr">
-        <is>
-          <t>2852.872</t>
-        </is>
+      <c r="D32" s="22" t="n">
+        <v>2567.5848</v>
       </c>
       <c r="E32" s="23" t="n"/>
       <c r="F32" s="23" t="n"/>
@@ -990,10 +976,8 @@
         </is>
       </c>
       <c r="C33" s="20" t="n"/>
-      <c r="D33" s="22" t="inlineStr">
-        <is>
-          <t>4224.918</t>
-        </is>
+      <c r="D33" s="22" t="n">
+        <v>3802.4262</v>
       </c>
       <c r="E33" s="23" t="n"/>
       <c r="F33" s="23" t="n"/>
@@ -1032,10 +1016,8 @@
         </is>
       </c>
       <c r="C35" s="20" t="n"/>
-      <c r="D35" s="22" t="inlineStr">
-        <is>
-          <t>888.897</t>
-        </is>
+      <c r="D35" s="22" t="n">
+        <v>800.0073</v>
       </c>
       <c r="E35" s="23" t="n"/>
       <c r="F35" s="23" t="n"/>
@@ -1053,10 +1035,8 @@
         </is>
       </c>
       <c r="C36" s="20" t="n"/>
-      <c r="D36" s="22" t="inlineStr">
-        <is>
-          <t>1006.036</t>
-        </is>
+      <c r="D36" s="22" t="n">
+        <v>905.4323999999999</v>
       </c>
       <c r="E36" s="23" t="n"/>
       <c r="F36" s="23" t="n"/>
@@ -1074,10 +1054,8 @@
         </is>
       </c>
       <c r="C37" s="20" t="n"/>
-      <c r="D37" s="22" t="inlineStr">
-        <is>
-          <t>1284.213</t>
-        </is>
+      <c r="D37" s="22" t="n">
+        <v>1155.7917</v>
       </c>
       <c r="E37" s="23" t="n"/>
       <c r="F37" s="23" t="n"/>
@@ -1095,10 +1073,8 @@
         </is>
       </c>
       <c r="C38" s="20" t="n"/>
-      <c r="D38" s="22" t="inlineStr">
-        <is>
-          <t>2133.396</t>
-        </is>
+      <c r="D38" s="22" t="n">
+        <v>1920.0564</v>
       </c>
       <c r="E38" s="23" t="n"/>
       <c r="F38" s="23" t="n"/>
@@ -1116,10 +1092,8 @@
         </is>
       </c>
       <c r="C39" s="20" t="n"/>
-      <c r="D39" s="22" t="inlineStr">
-        <is>
-          <t>2767.105</t>
-        </is>
+      <c r="D39" s="22" t="n">
+        <v>2490.3945</v>
       </c>
       <c r="E39" s="23" t="n"/>
       <c r="F39" s="23" t="n"/>
@@ -1137,10 +1111,8 @@
         </is>
       </c>
       <c r="C40" s="20" t="n"/>
-      <c r="D40" s="22" t="inlineStr">
-        <is>
-          <t>3528.424</t>
-        </is>
+      <c r="D40" s="22" t="n">
+        <v>3175.5816</v>
       </c>
       <c r="E40" s="23" t="n"/>
       <c r="F40" s="23" t="n"/>
@@ -1158,10 +1130,8 @@
         </is>
       </c>
       <c r="C41" s="20" t="n"/>
-      <c r="D41" s="22" t="inlineStr">
-        <is>
-          <t>4961.133</t>
-        </is>
+      <c r="D41" s="22" t="n">
+        <v>4465.0197</v>
       </c>
       <c r="E41" s="23" t="n"/>
       <c r="F41" s="23" t="n"/>
@@ -1179,10 +1149,8 @@
         </is>
       </c>
       <c r="C42" s="20" t="n"/>
-      <c r="D42" s="22" t="inlineStr">
-        <is>
-          <t>7655.029</t>
-        </is>
+      <c r="D42" s="22" t="n">
+        <v>6889.5261</v>
       </c>
       <c r="E42" s="23" t="n"/>
       <c r="F42" s="23" t="n"/>

</xml_diff>